<commit_message>
Refine the booking system
</commit_message>
<xml_diff>
--- a/booking/CIU-bookings-template.xlsx
+++ b/booking/CIU-bookings-template.xlsx
@@ -533,11 +533,11 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>45</v>
+        <v>1826</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>How many days ahead people can book</t>
+          <t>How many days ahead people can book (1826 = about 5 years)</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>tuadiel6@gmail.com</t>
+          <t>centreishemaryumuryango@gmail.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>TESTING: change to centre.ishemaryumuryango@yahoo.com before launch. Where new booking alerts are sent (comma-separate several)</t>
+          <t>Where new booking alerts are sent (comma-separate several)</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+250 788 733 368</t>
+          <t>+250 789 766 172</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Sample hours: replace with the centre's real hours. One row per opening period; 24-hour times (HH:MM). Leave out a day to close it every week.</t>
+          <t>Centre hours: Monday to Friday 07:00-20:00, Sunday 09:00-17:00. Saturday is a day off, so it has no row. 24-hour times (HH:MM).</t>
         </is>
       </c>
     </row>
@@ -656,92 +656,92 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>20:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>20:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>20:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -751,72 +751,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="6" t="n"/>

</xml_diff>